<commit_message>
Increased permutations for all datasets
</commit_message>
<xml_diff>
--- a/manuscript/robustness/Supplemental_Table_1.xlsx
+++ b/manuscript/robustness/Supplemental_Table_1.xlsx
@@ -16,11 +16,11 @@
     <sheet name="References" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'All Cell Types'!$A$1:$K$42</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Astrocytes!$A$1:$K$19</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Excitatory!$A$1:$K$24</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inhibitory!$A$1:$K$24</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Microglia!$A$1:$K$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'All Cell Types'!$A$1:$L$42</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Astrocytes!$A$1:$L$19</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Excitatory!$A$1:$L$24</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Inhibitory!$A$1:$L$24</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Microglia!$A$1:$L$21</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">References!$A$1:$C$54</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="441">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1354,6 +1354,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.nature.com/articles/s41467-026-68920-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">recurSieve adjusted p-value (BH)</t>
   </si>
 </sst>
 </file>
@@ -1900,7 +1903,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K1048576"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -1911,9 +1914,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1942,12 +1946,15 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1975,16 +1982,19 @@
         <v>1</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I2" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J2" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2012,16 +2022,19 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I3" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J3" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2049,16 +2062,19 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I4" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J4" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="K4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2086,16 +2102,19 @@
         <v>0.4</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I5" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J5" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2123,16 +2142,19 @@
         <v>1</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I6" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J6" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2160,16 +2182,19 @@
         <v>1</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I7" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2197,16 +2222,19 @@
         <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I8" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="s">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0534132360604481</v>
+      </c>
+      <c r="J8" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2234,16 +2262,19 @@
         <v>0.1</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I9" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="s">
+        <v>0.0594059405940594</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0608910891089108</v>
+      </c>
+      <c r="J9" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2271,16 +2302,19 @@
         <v>1</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I10" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J10" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>39</v>
       </c>
     </row>
@@ -2308,16 +2342,19 @@
         <v>1</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I11" s="6" t="b">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0534132360604481</v>
+      </c>
+      <c r="J11" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="K11" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2345,16 +2382,19 @@
         <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I12" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J12" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2382,16 +2422,19 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I13" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="8" t="s">
+        <v>0.0693069306930693</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0693069306930693</v>
+      </c>
+      <c r="J13" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2419,16 +2462,19 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I14" s="6" t="b">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J14" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="K14" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2456,16 +2502,19 @@
         <v>1</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I15" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J15" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2493,16 +2542,19 @@
         <v>1</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I16" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="s">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0534132360604481</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2530,16 +2582,19 @@
         <v>0.7</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I17" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J17" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2567,16 +2622,19 @@
         <v>0.5</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I18" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J18" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2604,16 +2662,19 @@
         <v>0.5</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I19" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J19" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2641,16 +2702,19 @@
         <v>1</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I20" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J20" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="L20" s="8" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2678,16 +2742,19 @@
         <v>1</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I21" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J21" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="L21" s="8" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2715,16 +2782,19 @@
         <v>1</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I22" s="6" t="b">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J22" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="K22" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="L22" s="8" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2752,16 +2822,19 @@
         <v>1</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.115384615384615</v>
-      </c>
-      <c r="I23" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J23" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="L23" s="8" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2789,16 +2862,19 @@
         <v>1</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I24" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J24" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K24" s="8" t="s">
+      <c r="L24" s="8" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2826,16 +2902,19 @@
         <v>1</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I25" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J25" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J25" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K25" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K25" s="8" t="s">
+      <c r="L25" s="8" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2863,16 +2942,19 @@
         <v>1</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I26" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J26" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K26" s="8" t="s">
+      <c r="L26" s="8" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2900,16 +2982,19 @@
         <v>1</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I27" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J27" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J27" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K27" s="8" t="s">
+      <c r="L27" s="8" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2937,16 +3022,19 @@
         <v>1</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I28" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J28" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K28" s="8" t="s">
+      <c r="L28" s="8" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2974,16 +3062,19 @@
         <v>1</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I29" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J29" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J29" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K29" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="K29" s="8" t="s">
+      <c r="L29" s="8" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3011,16 +3102,19 @@
         <v>1</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I30" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J30" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J30" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K30" s="8" t="s">
+      <c r="L30" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3048,16 +3142,19 @@
         <v>1</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I31" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J31" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J31" s="8" t="s">
+      <c r="K31" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="K31" s="8" t="s">
+      <c r="L31" s="8" t="s">
         <v>93</v>
       </c>
     </row>
@@ -3085,16 +3182,19 @@
         <v>0.9</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I32" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J32" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J32" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K32" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K32" s="8" t="s">
+      <c r="L32" s="8" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3122,16 +3222,19 @@
         <v>0.8</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I33" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J33" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K33" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K33" s="8" t="s">
+      <c r="L33" s="8" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3159,16 +3262,19 @@
         <v>1</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I34" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J34" s="8" t="s">
+        <v>0.0594059405940594</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0.0608910891089108</v>
+      </c>
+      <c r="J34" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K34" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K34" s="8" t="s">
+      <c r="L34" s="8" t="s">
         <v>99</v>
       </c>
     </row>
@@ -3196,16 +3302,19 @@
         <v>1</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I35" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J35" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K35" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K35" s="8" t="s">
+      <c r="L35" s="8" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3233,16 +3342,19 @@
         <v>0.5</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I36" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J36" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J36" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K36" s="8" t="s">
+      <c r="L36" s="8" t="s">
         <v>103</v>
       </c>
     </row>
@@ -3270,16 +3382,19 @@
         <v>0.8</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I37" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J37" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="K37" s="8" t="s">
+      <c r="L37" s="8" t="s">
         <v>106</v>
       </c>
     </row>
@@ -3307,16 +3422,19 @@
         <v>0.9</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I38" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J38" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J38" s="8" t="s">
+      <c r="K38" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K38" s="8" t="s">
+      <c r="L38" s="8" t="s">
         <v>108</v>
       </c>
     </row>
@@ -3344,16 +3462,19 @@
         <v>0.7</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I39" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J39" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K39" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K39" s="8" t="s">
+      <c r="L39" s="8" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3381,16 +3502,19 @@
         <v>0.4</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I40" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J40" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J40" s="8" t="s">
+      <c r="K40" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K40" s="8" t="s">
+      <c r="L40" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3418,16 +3542,19 @@
         <v>0.1</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I41" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J41" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0.0463932107496464</v>
+      </c>
+      <c r="J41" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K41" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="K41" s="8" t="s">
+      <c r="L41" s="8" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3455,22 +3582,25 @@
         <v>0.1</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I42" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J42" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.0434936350777934</v>
+      </c>
+      <c r="J42" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K42" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K42" s="8" t="s">
+      <c r="L42" s="8" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:K42"/>
+  <autoFilter ref="A1:L42"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3487,7 +3617,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -3498,9 +3628,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3529,12 +3660,15 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3562,16 +3696,19 @@
         <v>0.6</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I2" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J2" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3599,16 +3736,19 @@
         <v>0.9</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I3" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J3" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>120</v>
       </c>
     </row>
@@ -3636,16 +3776,19 @@
         <v>0.5</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.115384615384615</v>
-      </c>
-      <c r="I4" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J4" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>123</v>
       </c>
     </row>
@@ -3673,16 +3816,19 @@
         <v>0.8</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I5" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.0414041404140414</v>
+      </c>
+      <c r="J5" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3710,16 +3856,19 @@
         <v>0.9</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I6" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J6" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3747,16 +3896,19 @@
         <v>0.9</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I7" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>129</v>
       </c>
     </row>
@@ -3784,16 +3936,19 @@
         <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I8" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J8" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3821,16 +3976,19 @@
         <v>0.9</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I9" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J9" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3858,16 +4016,19 @@
         <v>0.9</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I10" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J10" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3895,16 +4056,19 @@
         <v>0.9</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I11" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="8" t="s">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="J11" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>132</v>
       </c>
     </row>
@@ -3932,16 +4096,19 @@
         <v>0.9</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I12" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J12" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="K12" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3969,16 +4136,19 @@
         <v>0.9</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I13" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J13" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4006,16 +4176,19 @@
         <v>0.9</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I14" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J14" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>137</v>
       </c>
     </row>
@@ -4043,16 +4216,19 @@
         <v>0.9</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I15" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J15" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>139</v>
       </c>
     </row>
@@ -4080,16 +4256,19 @@
         <v>0.8</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I16" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>141</v>
       </c>
     </row>
@@ -4117,16 +4296,19 @@
         <v>0.8</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I17" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J17" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>143</v>
       </c>
     </row>
@@ -4154,16 +4336,19 @@
         <v>0.4</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I18" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J18" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="K18" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4191,16 +4376,19 @@
         <v>0.7</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I19" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J19" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>145</v>
       </c>
     </row>
@@ -4228,16 +4416,19 @@
         <v>0.2</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I20" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J20" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="L20" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4265,16 +4456,19 @@
         <v>0.4</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I21" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J21" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="L21" s="8" t="s">
         <v>148</v>
       </c>
     </row>
@@ -4302,16 +4496,19 @@
         <v>0.4</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I22" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J22" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="L22" s="8" t="s">
         <v>150</v>
       </c>
     </row>
@@ -4339,16 +4536,19 @@
         <v>0.6</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I23" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.0267909143855562</v>
+      </c>
+      <c r="J23" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="L23" s="8" t="s">
         <v>153</v>
       </c>
     </row>
@@ -4376,21 +4576,24 @@
         <v>0.2</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I24" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0227722772277227</v>
+      </c>
+      <c r="J24" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="K24" s="8" t="s">
+      <c r="L24" s="8" t="s">
         <v>106</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K24"/>
+  <autoFilter ref="A1:L24"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4407,7 +4610,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -4418,9 +4621,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4449,12 +4653,15 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -4482,16 +4689,19 @@
         <v>0.8</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.115384615384615</v>
-      </c>
-      <c r="I2" s="6" t="b">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="J2" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4519,16 +4729,19 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I3" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J3" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4556,16 +4769,19 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I4" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J4" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="K4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>24</v>
       </c>
     </row>
@@ -4593,16 +4809,19 @@
         <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I5" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J5" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>159</v>
       </c>
     </row>
@@ -4630,16 +4849,19 @@
         <v>1</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I6" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J6" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -4667,16 +4889,19 @@
         <v>0.3</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I7" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>162</v>
       </c>
     </row>
@@ -4704,16 +4929,19 @@
         <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I8" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J8" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="K8" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>165</v>
       </c>
     </row>
@@ -4741,16 +4969,19 @@
         <v>1</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I9" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J9" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -4778,16 +5009,19 @@
         <v>1</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I10" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J10" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="K10" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -4815,16 +5049,19 @@
         <v>1</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I11" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J11" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4852,16 +5089,19 @@
         <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I12" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J12" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>168</v>
       </c>
     </row>
@@ -4889,16 +5129,19 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I13" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J13" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4926,16 +5169,19 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I14" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J14" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>145</v>
       </c>
     </row>
@@ -4963,16 +5209,19 @@
         <v>0.9</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I15" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J15" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>170</v>
       </c>
     </row>
@@ -5000,16 +5249,19 @@
         <v>0.9</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I16" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5037,16 +5289,19 @@
         <v>0.8</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I17" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J17" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="K17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5074,16 +5329,19 @@
         <v>0.8</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I18" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J18" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>174</v>
       </c>
     </row>
@@ -5111,16 +5369,19 @@
         <v>1</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I19" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J19" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>177</v>
       </c>
     </row>
@@ -5148,16 +5409,19 @@
         <v>0.7</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I20" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J20" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="L20" s="8" t="s">
         <v>179</v>
       </c>
     </row>
@@ -5185,16 +5449,19 @@
         <v>0.3</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I21" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J21" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="K21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="L21" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5222,16 +5489,19 @@
         <v>0.6</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I22" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J22" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="L22" s="8" t="s">
         <v>106</v>
       </c>
     </row>
@@ -5259,16 +5529,19 @@
         <v>0.8</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I23" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="J23" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="L23" s="8" t="s">
         <v>181</v>
       </c>
     </row>
@@ -5296,21 +5569,24 @@
         <v>0.4</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I24" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0325318246110325</v>
+      </c>
+      <c r="J24" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K24" s="8" t="s">
+      <c r="L24" s="8" t="s">
         <v>183</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K24"/>
+  <autoFilter ref="A1:L24"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5327,7 +5603,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -5338,9 +5614,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5369,12 +5646,15 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -5402,16 +5682,19 @@
         <v>1</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I2" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J2" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>186</v>
       </c>
     </row>
@@ -5439,16 +5722,19 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I3" s="6" t="b">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="J3" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>189</v>
       </c>
     </row>
@@ -5476,16 +5762,19 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I4" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J4" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -5513,16 +5802,19 @@
         <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I5" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J5" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>192</v>
       </c>
     </row>
@@ -5550,16 +5842,19 @@
         <v>1</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I6" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J6" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>195</v>
       </c>
     </row>
@@ -5587,16 +5882,19 @@
         <v>0.9</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I7" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>198</v>
       </c>
     </row>
@@ -5624,16 +5922,19 @@
         <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I8" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J8" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>201</v>
       </c>
     </row>
@@ -5661,16 +5962,19 @@
         <v>1</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I9" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J9" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -5698,16 +6002,19 @@
         <v>1</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I10" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J10" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>204</v>
       </c>
     </row>
@@ -5735,16 +6042,19 @@
         <v>0.6</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.115384615384615</v>
-      </c>
-      <c r="I11" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.0334158415841584</v>
+      </c>
+      <c r="J11" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -5772,16 +6082,19 @@
         <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I12" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J12" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="K12" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5809,16 +6122,19 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I13" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J13" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="K13" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>139</v>
       </c>
     </row>
@@ -5846,16 +6162,19 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I14" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J14" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>207</v>
       </c>
     </row>
@@ -5883,16 +6202,19 @@
         <v>1</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I15" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J15" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="K15" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5920,16 +6242,19 @@
         <v>1</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I16" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>211</v>
       </c>
     </row>
@@ -5957,16 +6282,19 @@
         <v>1</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I17" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="8" t="s">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.0396039603960396</v>
+      </c>
+      <c r="J17" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>213</v>
       </c>
     </row>
@@ -5994,16 +6322,19 @@
         <v>1</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I18" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.0254596888260254</v>
+      </c>
+      <c r="J18" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>177</v>
       </c>
     </row>
@@ -6031,21 +6362,24 @@
         <v>0.4</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I19" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0334158415841584</v>
+      </c>
+      <c r="J19" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="K19" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>137</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K19"/>
+  <autoFilter ref="A1:L19"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -6062,7 +6396,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -6073,9 +6407,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6104,12 +6439,15 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -6137,16 +6475,19 @@
         <v>1</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I2" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J2" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>216</v>
       </c>
     </row>
@@ -6174,16 +6515,19 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I3" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J3" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>219</v>
       </c>
     </row>
@@ -6211,16 +6555,19 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I4" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.034944670937682</v>
+      </c>
+      <c r="J4" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="K4" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>222</v>
       </c>
     </row>
@@ -6248,16 +6595,19 @@
         <v>1</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I5" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J5" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>189</v>
       </c>
     </row>
@@ -6285,16 +6635,19 @@
         <v>0.2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I6" s="6" t="b">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J6" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="K6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -6322,16 +6675,19 @@
         <v>0.2</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I7" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="s">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="J7" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>225</v>
       </c>
     </row>
@@ -6359,16 +6715,19 @@
         <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I8" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.034944670937682</v>
+      </c>
+      <c r="J8" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>228</v>
       </c>
     </row>
@@ -6396,16 +6755,19 @@
         <v>0.4</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I9" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.034944670937682</v>
+      </c>
+      <c r="J9" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>231</v>
       </c>
     </row>
@@ -6433,16 +6795,19 @@
         <v>1</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.115384615384615</v>
-      </c>
-      <c r="I10" s="6" t="b">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="J10" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="K10" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>234</v>
       </c>
     </row>
@@ -6470,16 +6835,19 @@
         <v>1</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I11" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J11" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -6507,16 +6875,19 @@
         <v>0.6</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I12" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J12" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -6544,16 +6915,19 @@
         <v>1</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I13" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J13" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="K13" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>172</v>
       </c>
     </row>
@@ -6581,16 +6955,19 @@
         <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I14" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J14" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>172</v>
       </c>
     </row>
@@ -6618,16 +6995,19 @@
         <v>0.5</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I15" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J15" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>238</v>
       </c>
     </row>
@@ -6655,16 +7035,19 @@
         <v>0.8</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I16" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="s">
+        <v>0.0099009900990099</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J16" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>139</v>
       </c>
     </row>
@@ -6692,16 +7075,19 @@
         <v>1</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.0384615384615384</v>
-      </c>
-      <c r="I17" s="6" t="b">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J17" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="K17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>240</v>
       </c>
     </row>
@@ -6729,16 +7115,19 @@
         <v>0.5</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I18" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="8" t="s">
+        <v>0.0198019801980198</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.033003300330033</v>
+      </c>
+      <c r="J18" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>242</v>
       </c>
     </row>
@@ -6766,16 +7155,19 @@
         <v>0.7</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I19" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="s">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.0495049504950495</v>
+      </c>
+      <c r="J19" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>112</v>
       </c>
     </row>
@@ -6803,16 +7195,19 @@
         <v>0.9</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I20" s="6" t="b">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.034944670937682</v>
+      </c>
+      <c r="J20" s="6" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="K20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="L20" s="8" t="s">
         <v>245</v>
       </c>
     </row>
@@ -6840,21 +7235,24 @@
         <v>0.4</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.0769230769230769</v>
-      </c>
-      <c r="I21" s="6" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="8" t="s">
+        <v>0.0297029702970297</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.034944670937682</v>
+      </c>
+      <c r="J21" s="6" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="L21" s="8" t="s">
         <v>247</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
+  <autoFilter ref="A1:L21"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>